<commit_message>
Undécima revisión: contraste en modo oscuro, CSS, avisos, diagramas de la base y documentos
- Web: rojo propio del modo oscuro, puntos y coma faltantes en styles.css,
  avisos largos que se salían de la pantalla, verde del tema en los mensajes.
- Base: comentarios de schema.sql corregidos y SQL completo regenerado.
- ERD y DER_Negocio: columna creado_por_invitado (migración 019), también
  dentro de la Documentación de Proyecto.
- Planillas: componentes de la placa completos (capacitor 470 µF y Nivel 2),
  checklist con los códigos de error del monitor serie.
- Word y LEEME: bobinas (cuatro, confirmado el 19/09), columnas 1 a 8,
  cantidades actualizadas, referencias inexistentes y marcas de comentario rotas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QiY8ZZNAM9gwPKiqSkCaaj
</commit_message>
<xml_diff>
--- a/documentacion_proyecto/Checklist_verificaciones.xlsx
+++ b/documentacion_proyecto/Checklist_verificaciones.xlsx
@@ -1073,12 +1073,12 @@
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>"Estado inicial sincronizado" y sin errores HTTP</t>
+          <t>"Estado inicial: ... (sin actuar)" y ningún "Error consultando estado"</t>
         </is>
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>404 = revisar TELAR_ID · error de conexión = despertar Render</t>
+          <t>HTTP 401 = DEVICE_KEY distinta de ESP32_DEVICE_KEY · 404 = revisar TELAR_ID · error de conexión = esperar a que despierte Render</t>
         </is>
       </c>
       <c r="G24" s="10" t="n"/>

</xml_diff>

<commit_message>
Segunda vuelta de revisión: textos, planillas, diagrama A y C y web
- Web: se quitan curCol y curPass, que ya no se usaban.
- Conexionado del Nivel 2 y guía de los Bloques C y D: la cinta se mueve a mano
  (Impulso está desconectado).
- Estimación de costos: celdas de la vida útil unidas, vida eléctrica del relé,
  4,75 V como mínimo de la fuente.
- Checklist de verificaciones: plaqueta principal en lugar de protoboard.
- Diagrama de los Bloques A y C: título (el sensor es del Nivel 2) y conexiones
  que ya no cruzan las cajas.
- Manual de instalación, autenticación, análisis del frontend, README del
  firmware y del backend, recomendaciones eléctricas y Nivel 2: datos al día.
- Migración 002: comentario de la posición al día (SQL completo regenerado).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QiY8ZZNAM9gwPKiqSkCaaj
</commit_message>
<xml_diff>
--- a/documentacion_proyecto/Checklist_verificaciones.xlsx
+++ b/documentacion_proyecto/Checklist_verificaciones.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Protoboard</t>
+          <t>Plaqueta principal</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
@@ -489,7 +489,7 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>Multímetro en continuidad, puntas en los dos rieles, todo desconectado</t>
+          <t>Multímetro en continuidad, puntas en +5 V y GND, todo desconectado</t>
         </is>
       </c>
       <c r="E3" s="10" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Capacitor</t>
+          <t>Capacitor de sensado</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>Capacitor</t>
+          <t>Capacitor de sensado</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>Continuidad entre una pata del capacitor y el riel GND</t>
+          <t>Continuidad entre una pata del capacitor y el GND del ESP32</t>
         </is>
       </c>
       <c r="E31" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Solo sensado y vista para los clientes con una clave por tejido
- Solo sensado: un interruptor en la barra del editor apaga el control
  del telar desde la página (sin pulsos de Marcha, Pausa ni Retroceder)
  y el sensado sigue. Migración 023, PUT /api/telares/:id/control-web,
  409 CONTROL_WEB_DESACTIVADO y el firmware que no pulsa los relés.
- Vista para clientes: cada dibujo puede tener una clave TEJ-XXXX-XXXX
  (hash + copia cifrada, migración 024). El cliente entra con ella y ve
  solo su tejido, sin ningún control. Rutas /api/cliente/* con cookie
  propia y límite de intentos fallidos.
- Pruebas, documentos (Word, PDF, Markdown, diagramas, checklist) y
  registro de cambios al día.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QiY8ZZNAM9gwPKiqSkCaaj
</commit_message>
<xml_diff>
--- a/documentacion_proyecto/Checklist_verificaciones.xlsx
+++ b/documentacion_proyecto/Checklist_verificaciones.xlsx
@@ -411,7 +411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="6" min="1" max="1"/>
@@ -900,7 +900,7 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Multímetro en modo diodo, entre + y −</t>
+          <t>Multímetro en modo diodo, entre + y −</t>
         </is>
       </c>
       <c r="E18" s="10" t="inlineStr">
@@ -1313,6 +1313,51 @@
       </c>
       <c r="G32" s="11" t="n"/>
     </row>
+    <row r="33" ht="23.85" customHeight="1" s="7">
+      <c r="A33" s="9" t="n"/>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>── CONTROL DESDE LA PÁGINA ──</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="n"/>
+      <c r="D33" s="9" t="n"/>
+      <c r="E33" s="9" t="n"/>
+      <c r="F33" s="9" t="n"/>
+      <c r="G33" s="9" t="n"/>
+    </row>
+    <row r="34" ht="40" customHeight="1" s="7">
+      <c r="A34" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>Solo sensado</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>Que con el control desde la página apagado no se mueva ningún relé</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>En la web, apagar «Control desde la página» y tocar ▶ (carga el dibujo), ⏸ y ⏪. Después volver a prenderlo</t>
+        </is>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>Ningún clic al apagarlo ni al tocar los botones, y tampoco al volver a prenderlo. La botonera sigue avisando</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>Si un relé hace clic, el firmware no es el actual: volver a cargarlo</t>
+        </is>
+      </c>
+      <c r="G34" s="10" t="n"/>
+    </row>
+    <row r="35" ht="28" customHeight="1" s="7"/>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Revisión ampliada, vuelta 1: estados viejos, letras sin formato y planillas cortadas
Textos que seguían en la etapa anterior (Árbol de docs/analisis, Bitácora,
Estimación, Modalidad, Conexionado, Parado automático), el texto alternativo
de nueve imágenes de los sitios, negritas y letras sin formato en el Estado
completo, la Guía C y D y la Estimación, filas de las planillas con texto
cortado y la Checklist, que se imprimía en 8 hojas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QiY8ZZNAM9gwPKiqSkCaaj
</commit_message>
<xml_diff>
--- a/documentacion_proyecto/Checklist_verificaciones.xlsx
+++ b/documentacion_proyecto/Checklist_verificaciones.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verificaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Verificaciones'!$1:$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
 </file>
@@ -123,7 +125,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -157,6 +159,15 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -409,7 +420,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
@@ -504,31 +515,31 @@
       </c>
       <c r="G3" s="10" t="n"/>
     </row>
-    <row r="4" ht="28" customHeight="1" s="7">
-      <c r="A4" s="10" t="n">
+    <row r="4" ht="36" customHeight="1" s="7">
+      <c r="A4" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Polarización</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>Que las resistencias de polarización estén en el nivel correcto</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Multímetro en VDC entre cada GPIO y GND, con el ESP32 alimentado</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="12" t="inlineStr">
         <is>
           <t>GPIO 25/26/32/33/34/35 ≈ 3,3 V · GPIO 27 ≈ 0 V · GPIO 18/19/21/22 ≈ 0 V (si el Bloque D ya está armado)</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr">
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>Si GPIO 27 da 3,3 V, su resistencia está a 3V3 y debe ir a GND</t>
         </is>
@@ -566,9 +577,9 @@
       </c>
       <c r="G5" s="10" t="n"/>
     </row>
-    <row r="6" ht="23.85" customHeight="1" s="7">
+    <row r="6" ht="26.25" customHeight="1" s="7">
       <c r="A6" s="9" t="n"/>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>── LÍNEA DE 220 V ──</t>
         </is>
@@ -579,31 +590,31 @@
       <c r="F6" s="9" t="n"/>
       <c r="G6" s="9" t="n"/>
     </row>
-    <row r="7" ht="15" customHeight="1" s="7">
-      <c r="A7" s="10" t="n">
+    <row r="7" ht="25" customHeight="1" s="7">
+      <c r="A7" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Fusible</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>Que el portafusible con el fusible haga contacto</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Multímetro en continuidad en los dos extremos del portafusible</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Debe pitar (0 Ω)</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr">
+      <c r="F7" s="12" t="inlineStr">
         <is>
           <t>Fusible mal encastrado o quemado</t>
         </is>
@@ -641,31 +652,31 @@
       </c>
       <c r="G8" s="10" t="n"/>
     </row>
-    <row r="9" ht="15" customHeight="1" s="7">
-      <c r="A9" s="10" t="n">
+    <row r="9" ht="25" customHeight="1" s="7">
+      <c r="A9" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Empalmes</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Que no quede cobre expuesto en la zona de 220 V</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Inspección visual</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Todo cubierto con termocontraíble o cinta</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F9" s="12" t="inlineStr">
         <is>
           <t>Aislar antes de enchufar</t>
         </is>
@@ -734,31 +745,31 @@
       </c>
       <c r="G11" s="10" t="n"/>
     </row>
-    <row r="12" ht="15" customHeight="1" s="7">
-      <c r="A12" s="10" t="n">
+    <row r="12" ht="25" customHeight="1" s="7">
+      <c r="A12" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>Identificar cuál par es la salida de 5 V</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>La medición anterior lo confirma</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="E12" s="12" t="inlineStr">
         <is>
           <t>El par que da 5 V es +Vo/−Vo</t>
         </is>
       </c>
-      <c r="F12" s="10" t="inlineStr">
+      <c r="F12" s="12" t="inlineStr">
         <is>
           <t>Si el que da 5 V es el otro par, el cableado está cruzado</t>
         </is>
@@ -809,62 +820,62 @@
       </c>
       <c r="G14" s="10" t="n"/>
     </row>
-    <row r="15" ht="28" customHeight="1" s="7">
-      <c r="A15" s="11" t="n">
+    <row r="15" ht="36" customHeight="1" s="7">
+      <c r="A15" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>Botonera</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr">
         <is>
           <t>CRÍTICO: sentido de la tensión en el botón</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="D15" s="14" t="inlineStr">
         <is>
           <t>Multímetro en VOLTAJE AC, telar encendido y sin tejer, puntas en los bornes del par NA</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>24 V en reposo y 0 V al apretar (así es el C 201: el ESP32 avisa cuando se suelta el botón)</t>
         </is>
       </c>
-      <c r="F15" s="11" t="inlineStr">
+      <c r="F15" s="14" t="inlineStr">
         <is>
           <t>Si da 0 V en reposo, ese no es el par NA (o es el NC): no conectar</t>
         </is>
       </c>
       <c r="G15" s="11" t="n"/>
     </row>
-    <row r="16" ht="40" customHeight="1" s="7">
-      <c r="A16" s="10" t="n">
+    <row r="16" ht="47" customHeight="1" s="7">
+      <c r="A16" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Botonera</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C16" s="12" t="inlineStr">
         <is>
           <t>Confirmar la tensión real</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>La misma medición</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="E16" s="12" t="inlineStr">
         <is>
           <t>Se espera 24 V en alterna (medido en el C 201 el 19/08/2026): anotar el valor</t>
         </is>
       </c>
-      <c r="F16" s="10" t="inlineStr">
+      <c r="F16" s="12" t="inlineStr">
         <is>
           <t>Si es 110/220 V, NO conectar. Con 18 a 24 V va la resistencia de 2,2 kΩ 1 W; con 12 a 18 V, la de 1,2 kΩ 1 W. El puente rectificador hace que funcione igual en alterna o continua</t>
         </is>
@@ -946,71 +957,71 @@
       </c>
       <c r="G19" s="10" t="n"/>
     </row>
-    <row r="20" ht="15" customHeight="1" s="7">
-      <c r="A20" s="10" t="n">
+    <row r="20" ht="25" customHeight="1" s="7">
+      <c r="A20" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>Capacitor</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C20" s="12" t="inlineStr">
         <is>
           <t>Polaridad del electrolítico</t>
         </is>
       </c>
-      <c r="D20" s="10" t="inlineStr">
+      <c r="D20" s="12" t="inlineStr">
         <is>
           <t>Inspección: la pata larga (o el lado sin franja) es el +</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="E20" s="12" t="inlineStr">
         <is>
           <t>Pata larga al + del DB157</t>
         </is>
       </c>
-      <c r="F20" s="10" t="inlineStr">
+      <c r="F20" s="12" t="inlineStr">
         <is>
           <t>Invertido puede explotar o dejar de filtrar</t>
         </is>
       </c>
       <c r="G20" s="10" t="n"/>
     </row>
-    <row r="21" ht="52" customHeight="1" s="7">
-      <c r="A21" s="10" t="n">
+    <row r="21" ht="58" customHeight="1" s="7">
+      <c r="A21" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>Canal completo</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="C21" s="12" t="inlineStr">
         <is>
           <t>Que un solo apretón genere UN solo evento</t>
         </is>
       </c>
-      <c r="D21" s="10" t="inlineStr">
+      <c r="D21" s="12" t="inlineStr">
         <is>
           <t>Monitor serie a 115200, telar encendido: apretar el botón al menos medio segundo y soltar. Después, con el telar tejiendo, medir GPIO 32 contra GND en el gabinete</t>
         </is>
       </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="E21" s="12" t="inlineStr">
         <is>
           <t>Un solo mensaje "alguien apretó..." al soltar. Tejiendo, GPIO 32 sigue en 0 V</t>
         </is>
       </c>
-      <c r="F21" s="10" t="inlineStr">
+      <c r="F21" s="12" t="inlineStr">
         <is>
           <t>Mensajes solos sin tocar nada = falta el capacitor de ese canal o está invertido · ninguno = el toque fue muy corto, o revisar DB157, PC817 y GPIO (sin tocar nada da 0 V) · GPIO 32 en 3,3 V tejiendo: avisame (el telar puentea Marcha mientras anda)</t>
         </is>
       </c>
       <c r="G21" s="10" t="n"/>
     </row>
-    <row r="22" ht="23.85" customHeight="1" s="7">
+    <row r="22" ht="26.25" customHeight="1" s="7">
       <c r="A22" s="9" t="n"/>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>── SISTEMA COMPLETO ──</t>
         </is>
@@ -1083,31 +1094,31 @@
       </c>
       <c r="G24" s="10" t="n"/>
     </row>
-    <row r="25" ht="15" customHeight="1" s="7">
-      <c r="A25" s="10" t="n">
+    <row r="25" ht="25" customHeight="1" s="7">
+      <c r="A25" s="12" t="n">
         <v>19</v>
       </c>
-      <c r="B25" s="10" t="inlineStr">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>Órdenes web</t>
         </is>
       </c>
-      <c r="C25" s="10" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>Que los 3 relés respondan</t>
         </is>
       </c>
-      <c r="D25" s="10" t="inlineStr">
+      <c r="D25" s="12" t="inlineStr">
         <is>
           <t>Desde la web: ▶ Marcha, ⏸ Pausa, ⏪ Retroceder</t>
         </is>
       </c>
-      <c r="E25" s="10" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>Un clic corto por orden, hasta 2,5 s de demora</t>
         </is>
       </c>
-      <c r="F25" s="10" t="inlineStr">
+      <c r="F25" s="12" t="inlineStr">
         <is>
           <t>Si no responde, revisar el GPIO de ese canal</t>
         </is>
@@ -1145,9 +1156,9 @@
       </c>
       <c r="G26" s="10" t="n"/>
     </row>
-    <row r="27" ht="23.85" customHeight="1" s="7">
+    <row r="27" ht="26.25" customHeight="1" s="7">
       <c r="A27" s="9" t="n"/>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>── CABLEADO AL TELAR ──</t>
         </is>
@@ -1220,31 +1231,31 @@
       </c>
       <c r="G29" s="10" t="n"/>
     </row>
-    <row r="30" ht="15" customHeight="1" s="7">
-      <c r="A30" s="10" t="n">
+    <row r="30" ht="25" customHeight="1" s="7">
+      <c r="A30" s="12" t="n">
         <v>23</v>
       </c>
-      <c r="B30" s="10" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>Capacitor de sensado</t>
         </is>
       </c>
-      <c r="C30" s="10" t="inlineStr">
+      <c r="C30" s="12" t="inlineStr">
         <is>
           <t>Que no esté en corto</t>
         </is>
       </c>
-      <c r="D30" s="10" t="inlineStr">
+      <c r="D30" s="12" t="inlineStr">
         <is>
           <t>Multímetro en continuidad entre sus dos patas</t>
         </is>
       </c>
-      <c r="E30" s="10" t="inlineStr">
+      <c r="E30" s="12" t="inlineStr">
         <is>
           <t>NO debe pitar</t>
         </is>
       </c>
-      <c r="F30" s="10" t="inlineStr">
+      <c r="F30" s="12" t="inlineStr">
         <is>
           <t>Capacitor en corto: descartarlo</t>
         </is>
@@ -1313,9 +1324,9 @@
       </c>
       <c r="G32" s="11" t="n"/>
     </row>
-    <row r="33" ht="23.85" customHeight="1" s="7">
+    <row r="33" ht="26.25" customHeight="1" s="7">
       <c r="A33" s="9" t="n"/>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>── CONTROL DESDE LA PÁGINA ──</t>
         </is>
@@ -1361,6 +1372,6 @@
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualización al 28/10/2026: prueba completa del Nivel 2 y plaqueta del ESP32
- Gantt (desde la planilla de Drive), diagrama y PNG al 28/10.
- Registro de entrevistas: reunión del 28/10 con los dos videos.
- Bitácora: entradas del 22, 25, 26, 27 y 28/10.
- Plaqueta del ESP32 (PCB en PNG, SVG y DXF) y diagrama de plaquetas con
  los puentes de alambre.
- Lista de componentes, componentes en placa y checklist con lo usado de
  verdad.
- Estimación de costos y modalidad de contrato recalculadas, con el
  diagrama nuevo.
- Guías de conexión y puesta en marcha, mediciones y conexiones de las
  plaquetas con la plaqueta del ESP32 y lo medido el 28/10.
- Documentación de Proyecto (versión 5.2), estado completo, manual del
  telar, Nivel 2, árbol de problemas y Markdown al día.
- PDF regenerados. El firmware queda sin cambios.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QiY8ZZNAM9gwPKiqSkCaaj
</commit_message>
<xml_diff>
--- a/documentacion_proyecto/Checklist_verificaciones.xlsx
+++ b/documentacion_proyecto/Checklist_verificaciones.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="6" min="1" max="1"/>
@@ -1368,7 +1368,297 @@
       </c>
       <c r="G34" s="10" t="n"/>
     </row>
-    <row r="35" ht="28" customHeight="1" s="7"/>
+    <row r="35" ht="26.25" customHeight="1" s="7">
+      <c r="A35" s="9" t="n"/>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>── PLAQUETA DEL ESP32 ──</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="n"/>
+      <c r="D35" s="9" t="n"/>
+      <c r="E35" s="9" t="n"/>
+      <c r="F35" s="9" t="n"/>
+      <c r="G35" s="9" t="n"/>
+    </row>
+    <row r="36" ht="40" customHeight="1" s="7">
+      <c r="A36" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>Plaqueta del ESP32</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>Que cada cable de P1 y P2 llegue a su pad de la principal</t>
+        </is>
+      </c>
+      <c r="D36" s="10" t="inlineStr">
+        <is>
+          <t>Multímetro en continuidad, sin el ESP32 y sin alimentar, con la lista del punto 4.6 de la guía de conexión</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>Pita en cada cable, y no contra el pad de al lado</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="inlineStr">
+        <is>
+          <t>Cable en el pad equivocado: corregirlo antes de enchufar el ESP32</t>
+        </is>
+      </c>
+      <c r="G36" s="10" t="n"/>
+    </row>
+    <row r="37" ht="40" customHeight="1" s="7">
+      <c r="A37" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>Puentes de alambre</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>Que los tres puentes conecten</t>
+        </is>
+      </c>
+      <c r="D37" s="10" t="inlineStr">
+        <is>
+          <t>Continuidad de punta a punta: J4-3 ↔ J5-5 y J8-1 ↔ J5-6 en la principal; U3 ↔ R7 en la del Nivel 2</t>
+        </is>
+      </c>
+      <c r="E37" s="10" t="inlineStr">
+        <is>
+          <t>Pita en los tres, y no contra las patas de al lado</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="inlineStr">
+        <is>
+          <t>Rehacer ese puente</t>
+        </is>
+      </c>
+      <c r="G37" s="10" t="n"/>
+    </row>
+    <row r="38" ht="40" customHeight="1" s="7">
+      <c r="A38" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>Plaqueta del ESP32</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>La alimentación, antes de enchufar el ESP32</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="inlineStr">
+        <is>
+          <t>Multímetro en VDC, con la principal alimentada y sin el ESP32</t>
+        </is>
+      </c>
+      <c r="E38" s="10" t="inlineStr">
+        <is>
+          <t>5 V entre P1-10 y P1-9; 0 V en P1-1 (los 3,3 V los genera el ESP32)</t>
+        </is>
+      </c>
+      <c r="F38" s="10" t="inlineStr">
+        <is>
+          <t>5 V en otro pin: hay un cable cruzado. No enchufar el ESP32</t>
+        </is>
+      </c>
+      <c r="G38" s="10" t="n"/>
+    </row>
+    <row r="39" ht="26.25" customHeight="1" s="7">
+      <c r="A39" s="9" t="n"/>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>── NIVEL 2 (SENSOR Y RELÉS) ──</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="n"/>
+      <c r="D39" s="9" t="n"/>
+      <c r="E39" s="9" t="n"/>
+      <c r="F39" s="9" t="n"/>
+      <c r="G39" s="9" t="n"/>
+    </row>
+    <row r="40" ht="40" customHeight="1" s="7">
+      <c r="A40" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>Sensor de pasada</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>Que cuente una pasada por vuelta</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>Tejer 50 pasadas contadas a mano y compararlas con la web</t>
+        </is>
+      </c>
+      <c r="E40" s="10" t="inlineStr">
+        <is>
+          <t>La web suma 50</t>
+        </is>
+      </c>
+      <c r="F40" s="10" t="inlineStr">
+        <is>
+          <t>De más: rebote o eje equivocado · de menos: distancia al blanco (2 a 3 mm) o soporte</t>
+        </is>
+      </c>
+      <c r="G40" s="10" t="n"/>
+    </row>
+    <row r="41" ht="40" customHeight="1" s="7">
+      <c r="A41" s="10" t="n">
+        <v>31</v>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>Aislamiento</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>Que el lado del telar no toque el GND del ESP32</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>Continuidad entre el GND del ESP32 y los bornes de B2 y B3</t>
+        </is>
+      </c>
+      <c r="E41" s="10" t="inlineStr">
+        <is>
+          <t>NO debe pitar</t>
+        </is>
+      </c>
+      <c r="F41" s="10" t="inlineStr">
+        <is>
+          <t>Hay una unión entre los dos lados: encontrarla</t>
+        </is>
+      </c>
+      <c r="G41" s="10" t="n"/>
+    </row>
+    <row r="42" ht="40" customHeight="1" s="7">
+      <c r="A42" s="10" t="n">
+        <v>32</v>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>Relés LCA110</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>Que cada canal mueva su bobina</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>Tejer un dibujo con una sola columna marcada, de a una</t>
+        </is>
+      </c>
+      <c r="E42" s="10" t="inlineStr">
+        <is>
+          <t>Solo se activa la bobina de esa columna (canal 1 = GPIO 18 = bobina 1, y así)</t>
+        </is>
+      </c>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
+          <t>Se activa otra: cables cruzados en B3 (el 28/10/2026 pasó con los canales 2 y 3)</t>
+        </is>
+      </c>
+      <c r="G42" s="10" t="n"/>
+    </row>
+    <row r="43" ht="40" customHeight="1" s="7">
+      <c r="A43" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>Tejido</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>Que la tela salga como el dibujo</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>Tejer un tramo corto con franjas de colores y repeticiones distintas</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="inlineStr">
+        <is>
+          <t>Igual que en la web</t>
+        </is>
+      </c>
+      <c r="F43" s="10" t="inlineStr">
+        <is>
+          <t>Corrida una pasada: DESPLAZAMIENTO_FILAS · pasadas sin selección: PORCENTAJE_SELECCION</t>
+        </is>
+      </c>
+      <c r="G43" s="10" t="n"/>
+    </row>
+    <row r="44" ht="40" customHeight="1" s="7">
+      <c r="A44" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>Conteo</t>
+        </is>
+      </c>
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>Validar el conteo en una jornada</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="inlineStr">
+        <is>
+          <t>Anotar el contador mecánico del telar al empezar y al terminar el turno</t>
+        </is>
+      </c>
+      <c r="E44" s="10" t="inlineStr">
+        <is>
+          <t>Menos de 0,1 % de diferencia: tocar Validar en la web</t>
+        </is>
+      </c>
+      <c r="F44" s="10" t="inlineStr">
+        <is>
+          <t>Revisar soporte, distancia y cableado, y repetir</t>
+        </is>
+      </c>
+      <c r="G44" s="10" t="n"/>
+    </row>
+    <row r="45" ht="26.25" customHeight="1" s="7">
+      <c r="A45" s="9" t="n"/>
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>── PRUEBA DEL 28/10/2026 ──</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Verificaciones 1 a 33 bien. La 34 sigue en el período de prueba, hasta el 04/11/2026.</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="n"/>
+      <c r="E45" s="9" t="n"/>
+      <c r="F45" s="9" t="n"/>
+      <c r="G45" s="9" t="n"/>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
La prueba con las plaquetas fue el 30/10 y el precio final por telar
- 28/10 → 30/10 en READMEs, guías, Word, planillas y sus PDF (la prueba del
  proyecto completo, la reunión 8 y la entrada de la Bitácora).
- Gantt bajado de Drive con las tareas 7.7 a 7.11 y 8.17 desde el 30/10.
- Estimación de Costos: costos varios de $77.050 (insumos y dos meses de
  Claude Pro), inversión de $32.021.188 y precio final de $3.200.000 por
  telar, que la recupera con 19 telares en dos años.
- Modalidad, Documentación de Proyecto, Bitácora y el diagrama de costos
  con el precio por telar.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QiY8ZZNAM9gwPKiqSkCaaj
</commit_message>
<xml_diff>
--- a/documentacion_proyecto/Checklist_verificaciones.xlsx
+++ b/documentacion_proyecto/Checklist_verificaciones.xlsx
@@ -1575,7 +1575,7 @@
       </c>
       <c r="F42" s="10" t="inlineStr">
         <is>
-          <t>Se activa otra: cables cruzados en B3 (el 28/10/2026 pasó con los canales 2 y 3)</t>
+          <t>Se activa otra: cables cruzados en B3 (el 30/10/2026 pasó con los canales 2 y 3)</t>
         </is>
       </c>
       <c r="G42" s="10" t="n"/>
@@ -1646,7 +1646,7 @@
       <c r="A45" s="9" t="n"/>
       <c r="B45" s="13" t="inlineStr">
         <is>
-          <t>── PRUEBA DEL 28/10/2026 ──</t>
+          <t>── PRUEBA DEL 30/10/2026 ──</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">

</xml_diff>